<commit_message>
feat(arkusz-mapa): improve subcontractor list loading from XLSX
</commit_message>
<xml_diff>
--- a/docs/podwyko lista.xlsx
+++ b/docs/podwyko lista.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>Nazwa</t>
   </si>
@@ -173,6 +173,18 @@
   </si>
   <si>
     <t>THOR Recycle Sp. z o.o. NIP: 9452260589 BDO: 000575610</t>
+  </si>
+  <si>
+    <t>TARGET SPEED</t>
+  </si>
+  <si>
+    <t>TARGET SPEED SP. Z O.O., Braniborska 7/2, 53-680 Wrocław, NIP: 8971890822</t>
+  </si>
+  <si>
+    <t>P.M.C. Auto</t>
+  </si>
+  <si>
+    <t>P.M.C. Auto Lubuska 15, 09-408 Płock</t>
   </si>
 </sst>
 </file>
@@ -1073,8 +1085,12 @@
       <c r="Z19" s="1"/>
     </row>
     <row r="20" ht="14.25" customHeight="1">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
+      <c r="A20" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>39</v>
+      </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
@@ -1101,8 +1117,12 @@
       <c r="Z20" s="1"/>
     </row>
     <row r="21" ht="14.25" customHeight="1">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
+      <c r="A21" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>

</xml_diff>

<commit_message>
chore(arkusz-mapa): regenerate podwyko lista.ods from xlsx
</commit_message>
<xml_diff>
--- a/docs/podwyko lista.xlsx
+++ b/docs/podwyko lista.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>Nazwa</t>
   </si>
@@ -181,10 +181,16 @@
     <t>TARGET SPEED SP. Z O.O., Braniborska 7/2, 53-680 Wrocław, NIP: 8971890822</t>
   </si>
   <si>
-    <t>P.M.C. Auto</t>
+    <t>P.M.C. Auto (PLOMAT)</t>
   </si>
   <si>
-    <t>P.M.C. Auto Lubuska 15, 09-408 Płock</t>
+    <t>PLOMAT SP. z O.O.  Lubuska 15, 09-408 Płock BDO: 000719289 NIP: 7743231982</t>
+  </si>
+  <si>
+    <t>Wiślanka</t>
+  </si>
+  <si>
+    <t>Wiślanka Sp. z O.O. ul.Malinka 41C, 43-460 Wisła BDO: 000577060 NIP: 5482668086</t>
   </si>
 </sst>
 </file>
@@ -1149,8 +1155,12 @@
       <c r="Z21" s="1"/>
     </row>
     <row r="22" ht="14.25" customHeight="1">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
+      <c r="A22" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>43</v>
+      </c>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>

</xml_diff>

<commit_message>
chore(docs): add ECOLUX to subcontractor list
Sync podwyko lista.xlsx with updated ODS so the map uses the new carrier in the Word protocol dropdown.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/podwyko lista.xlsx
+++ b/docs/podwyko lista.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -607,9 +607,17 @@
         <v>GEODIS Poland Sp. z o.o., Wodna 38, 95-010 - Dobra</v>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>ECOLUX</v>
+      </c>
+      <c r="B27" t="str">
+        <v>ECOLUX ul. Handlowa 6a, 37-716 Orły NIP:7952458856 REGON:522494593</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B26"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(podwyko): add IWO SORTOWNIA ODPADÓW SEGREGOWANYCH to carrier list
</commit_message>
<xml_diff>
--- a/docs/podwyko lista.xlsx
+++ b/docs/podwyko lista.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -647,9 +647,17 @@
         <v>PHU SUDOWSCY D. SUDOWSKA W. SUDOWSKI S.C. BDO:000082474</v>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>IWO SORTOWNIA ODPADÓW SEGREGOWANYCH</v>
+      </c>
+      <c r="B32" t="str">
+        <v>IWO ul. Bielska 41, 17-120 Brańsk</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>